<commit_message>
updated the codes to return comparison of prodiction rates
</commit_message>
<xml_diff>
--- a/Data/HDC/HDC1_metabolomics_preliminary_formodelling2.xlsx
+++ b/Data/HDC/HDC1_metabolomics_preliminary_formodelling2.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - smail.iitm.ac.in\noor_com_model\Data\HDC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - smail.iitm.ac.in\noor_com_model\community_modelling\Data\HDC\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16515" windowHeight="7920"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16515" windowHeight="7920" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="consumed" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="172">
   <si>
     <t>Quantified compounds</t>
   </si>
@@ -549,9 +549,6 @@
   </si>
   <si>
     <t>HDC1_Mean (mmol per g)</t>
-  </si>
-  <si>
-    <t>HDC_1Standard deviation (mmol per g)</t>
   </si>
   <si>
     <t>HDC1_Standard deviation (mmol per g)</t>
@@ -598,13 +595,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -955,16 +949,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -977,9 +971,9 @@
         <v>170</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I1" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1396,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -1411,16 +1405,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1464,7 +1458,9 @@
       <c r="H2">
         <v>5.3274277260539362E-5</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
@@ -2594,15 +2590,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
-      <c r="I42" t="s">
-        <v>52</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="I1:I2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>